<commit_message>
Route-building: enforce co-occupancy limits from xlsx 'limitation' table
Encode the new 'cant happen' rows (E1<->P23, E1<->P24) as a declarative
CANT_COEXIST table (single source of truth, mirrors car position.xlsx).
Derive the block-2 aisle-clear condition from it (replacing the hardcoded
b[A1]===0), and add a general per-state validity guard to both A* solvers
so no route passes through a forbidden co-occupancy. Documented in
doc/ALGORITHMS.md.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/car position.xlsx
+++ b/car position.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boaze\Ai-Projects\parking systems\rotem-shani\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Aiprojects\parking systems\rotem shani\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6459E8F3-DB5D-4ECF-B3D8-0FB7B047B6AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{052D8D9C-F966-4DDD-89D6-36BAFF454993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4D0CD031-A119-4625-9AF9-4C97AA6C48F5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{4D0CD031-A119-4625-9AF9-4C97AA6C48F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="43">
   <si>
     <t>Parking Number</t>
   </si>
@@ -162,6 +162,12 @@
   </si>
   <si>
     <t>Opposite parking P1</t>
+  </si>
+  <si>
+    <t>limitation</t>
+  </si>
+  <si>
+    <t>cant happen</t>
   </si>
 </sst>
 </file>
@@ -571,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F29CA4C-52C3-4F9A-87A1-F53221D74662}">
-  <dimension ref="D3:AC32"/>
+  <dimension ref="D3:AC36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="13.28515625" customWidth="1"/>
@@ -1041,6 +1047,33 @@
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
     </row>
+    <row r="34" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D34" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="35" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D35" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D36" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Car 1: flip default orientation to face lift; route via E3; add intake motion
- rotem_saved.json: car 1 initial rot 97.3 -> 277.3 (faces the lift).
- MOVE_GRAPH (xlsx update): P1 connects only to E3; E3 -> {EL, W1, P1};
  E4 dropped from car 1's route (kept symmetric).
- car1Descent/car1Ascent + car1Cycle: car 1 rises/descends via E3, spins
  180 deg at W1, and parks at P1 facing the lift. Trigger: enter "1" +
  run extract.
- Earlier this session: top-view default + wider initial framing.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/car position.xlsx
+++ b/car position.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Aiprojects\parking systems\rotem shani\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{052D8D9C-F966-4DDD-89D6-36BAFF454993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB362128-FC11-4441-82DF-5868A2217860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{4D0CD031-A119-4625-9AF9-4C97AA6C48F5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="43">
   <si>
     <t>Parking Number</t>
   </si>
@@ -674,7 +674,9 @@
       <c r="G7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H7" s="3"/>
+      <c r="H7" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="I7" s="3"/>
     </row>
     <row r="8" spans="4:9" x14ac:dyDescent="0.25">
@@ -731,7 +733,7 @@
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>

</xml_diff>

<commit_message>
Constraint table: remove stale E4->P1 edge (E4 now connects to EL only)
xlsx now fully consistent with the code MOVE_GRAPH (P1<->E3 only; E4<->EL).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/car position.xlsx
+++ b/car position.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Aiprojects\parking systems\rotem shani\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB362128-FC11-4441-82DF-5868A2217860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4AEDA4F-855C-4B68-AC80-AF63906D9407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{4D0CD031-A119-4625-9AF9-4C97AA6C48F5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="43">
   <si>
     <t>Parking Number</t>
   </si>
@@ -702,9 +702,7 @@
       <c r="E9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>36</v>
-      </c>
+      <c r="F9" s="3"/>
       <c r="G9" s="3" t="s">
         <v>9</v>
       </c>

</xml_diff>